<commit_message>
feat(import): update Entry Transactions import template
</commit_message>
<xml_diff>
--- a/public/EntryTransactions_Import_Template.xlsx
+++ b/public/EntryTransactions_Import_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TaNtAwIi\Downloads\Alogorizm Level 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BD7E4E-01E7-4D5C-B430-921CD061CAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C36F23-A4A4-44DC-A30A-B40F8896E640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5052" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entry Transactions" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="101">
   <si>
     <t>IGNORE</t>
   </si>
@@ -315,13 +315,22 @@
   </si>
   <si>
     <t>User who created the record (default: Import)</t>
+  </si>
+  <si>
+    <t>GuideName</t>
+  </si>
+  <si>
+    <t>GuideDuty</t>
+  </si>
+  <si>
+    <t>GuideCostEGP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,6 +365,16 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="14">
@@ -426,7 +445,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -449,11 +468,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="22"/>
+      </left>
+      <right style="thin">
+        <color indexed="22"/>
+      </right>
+      <top style="thin">
+        <color indexed="22"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="22"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -530,9 +565,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal_Entry Transactions" xfId="1" xr:uid="{0A40B87F-603E-45E0-B474-EDFD7AF43261}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -832,8 +877,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BE3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:BG3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -860,9 +905,11 @@
     <col min="54" max="54" width="10" customWidth="1"/>
     <col min="55" max="55" width="14" customWidth="1"/>
     <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="57" width="17.42578125" customWidth="1"/>
+    <col min="58" max="59" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:59" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -877,7 +924,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="J1" s="3" t="s">
@@ -955,8 +1002,11 @@
       <c r="BD1" s="10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:57" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BE1" s="2"/>
+      <c r="BF1" s="2"/>
+      <c r="BG1" s="2"/>
+    </row>
+    <row r="2" spans="1:59" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>12</v>
       </c>
@@ -981,7 +1031,7 @@
       <c r="H2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="13" t="s">
         <v>20</v>
       </c>
       <c r="J2" s="13" t="s">
@@ -1125,27 +1175,36 @@
       <c r="BD2" s="20" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="3" spans="1:57" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BE2" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="BF2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="BG2" s="12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:59" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21"/>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
       <c r="T3" s="22"/>
       <c r="U3" s="22"/>
       <c r="V3" s="22"/>
@@ -1184,6 +1243,8 @@
       <c r="BC3" s="22"/>
       <c r="BD3" s="22"/>
       <c r="BE3" s="22"/>
+      <c r="BF3" s="22"/>
+      <c r="BG3" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1193,13 +1254,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>68</v>
       </c>
@@ -1207,7 +1268,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
         <v>12</v>
       </c>
@@ -1215,7 +1276,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>71</v>
       </c>
@@ -1223,7 +1284,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
         <v>73</v>
       </c>
@@ -1231,7 +1292,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>75</v>
       </c>
@@ -1239,7 +1300,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
         <v>16</v>
       </c>
@@ -1247,7 +1308,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>17</v>
       </c>
@@ -1255,7 +1316,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="24" t="s">
         <v>18</v>
       </c>
@@ -1263,7 +1324,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
         <v>19</v>
       </c>
@@ -1271,7 +1332,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
         <v>79</v>
       </c>
@@ -1279,7 +1340,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
         <v>21</v>
       </c>
@@ -1287,7 +1348,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
         <v>22</v>
       </c>
@@ -1295,7 +1356,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
         <v>82</v>
       </c>
@@ -1303,7 +1364,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
         <v>84</v>
       </c>
@@ -1311,7 +1372,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
         <v>86</v>
       </c>
@@ -1319,7 +1380,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
         <v>28</v>
       </c>
@@ -1327,7 +1388,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
         <v>29</v>
       </c>
@@ -1335,7 +1396,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>87</v>
       </c>
@@ -1343,7 +1404,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>89</v>
       </c>
@@ -1351,7 +1412,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
         <v>91</v>
       </c>
@@ -1359,7 +1420,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
         <v>60</v>
       </c>
@@ -1367,7 +1428,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="24" t="s">
         <v>61</v>
       </c>
@@ -1375,7 +1436,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
         <v>65</v>
       </c>
@@ -1383,7 +1444,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
         <v>66</v>
       </c>
@@ -1391,7 +1452,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
         <v>67</v>
       </c>

</xml_diff>